<commit_message>
Therapy Timeline: correct DKA-HYPOK-01 boxes B3/B7/B8/B11 after full-text check
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ZrxDdhKdHt6N5Ksq6Z7E7
</commit_message>
<xml_diff>
--- a/Therapy_Timeline_Cases.xlsx
+++ b/Therapy_Timeline_Cases.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Paper has: potassium unit mg/L vs mEq/L; weight 88.6 vs 88.4 kg; insulin threshold '&gt;3.3' vs 'achieved 3.3'. Resolve against the full text and do not guess.</t>
+          <t>Paper has: potassium unit mg/L vs mEq/L; weight 88.6 vs 88.4 kg; insulin threshold '&gt;3.3' vs 'achieved 3.3'. Resolve against the full text and do not guess. | First-pass check 20 Oct 2026: B3/B7/B8/B11 corrected against full text; B4 (250 mEq bicarbonate timing) and table-only values (K at 5/25/29/32/40 h, Mg 1.9) still need a teacher to check Table 1.</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -5434,12 +5434,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>IV potassium chloride + normal saline</t>
+          <t>IV potassium (salt not named)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>KCl 50 mEq and NaCl 1000 mL</t>
+          <t>50 mEq IV K (saline volume NOT STATED IN PAPER)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -5454,12 +5454,12 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Treatment timeline, 0 h</t>
+          <t>Case presentation text</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>(entered by hand; add exact quote when verifying)</t>
+          <t>initial repletion with 50 mEq of IV K resulted in only a slight increase from 3.0 to 3.1 mEq/L</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5635,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Insulin 4 U/h; KCl 40 mEq; K-Phos 30 mmol</t>
+          <t>Insulin infusion initiated (rate for this step NOT STATED IN PAPER); IV K replacement ongoing (Table 1 amounts KCl 40 mEq, K-Phos 30 mmol - table value, unverified)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>(entered by hand; add exact quote when verifying)</t>
+          <t>an insulin infusion was initiated with IV ongoing K replacement</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>CVVH potassium dialysate 4.0 mEq/L; insulin dose NOT STATED IN PAPER; bicarbonate content NOT STATED IN PAPER</t>
+          <t>CVVH with 4.0 mEq/L K dialysate and 40 mEq/L bicarbonate dialysate; insulin 4 U/h (88.6 kg patient)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -5700,12 +5700,12 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Text / Discussion</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>(entered by hand; add exact quote when verifying)</t>
+          <t>we chose to use a dialysate solution with bicarbonate content of 40 mEq/L ... while using a lower dose insulin infusion—4 U/h for this 88.6 kg patient</t>
         </is>
       </c>
     </row>
@@ -5841,12 +5841,12 @@
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>NOT STATED IN PAPER (interpretation)</t>
+          <t>PAPER</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>PAPER</t>
+          <t>Arrival Mg: case text. Fall to 1.9 mg/dL at 32 h: Table 1 only, unverified</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Therapy Timeline: mark 5 checked cases VERIFIED (ENDO-02, ID-01, ONC-01, RESP-01, RESP-02)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ZrxDdhKdHt6N5Ksq6Z7E7
</commit_message>
<xml_diff>
--- a/Therapy_Timeline_Cases.xlsx
+++ b/Therapy_Timeline_Cases.xlsx
@@ -1133,7 +1133,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Cardiovascular Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Cardiovascular Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Cardiovascular Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Cardiovascular Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1354,7 +1354,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Anara AI full-text check 2026-10-21; accepted by Dr. Hamdar</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1406,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1421,7 +1426,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Anara AI full-text check 2026-10-21; accepted by Dr. Hamdar</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1478,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1535,7 +1545,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Cureus publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1555,7 +1565,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Anara AI full-text check 2026-10-21; accepted by Dr. Hamdar</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1617,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1622,7 +1637,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Anara AI full-text check 2026-10-21; accepted by Dr. Hamdar</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1689,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
+          <t>CC BY - reported CONFIRMED on article page by Anara check (2026-10-21), accepted by Dr. Hamdar; not independently re-checked by Claude | prior: CC BY (journal policy: Frontiers in Medicine publishes all articles under CC BY 4.0) - NOT machine-verified, confirm on article page</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1689,7 +1709,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Anara AI full-text check 2026-10-21; accepted by Dr. Hamdar</t>
         </is>
       </c>
     </row>

</xml_diff>